<commit_message>
Need to implement cosmos
</commit_message>
<xml_diff>
--- a/About services.xlsx
+++ b/About services.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PK\E-Commerce\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED8A5B8-7F89-455C-B099-A1895B2C14E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3D64E77-6ACF-4C9B-992F-990F67DE9D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>Packages</t>
   </si>
@@ -78,6 +78,12 @@
   </si>
   <si>
     <t>Aspnetcore.OpenApi , EntityFrameworkCore.Design, Swashbuckle.Aspnetcore</t>
+  </si>
+  <si>
+    <t>Packages and its uses</t>
+  </si>
+  <si>
+    <t>Azure steps and role access</t>
   </si>
 </sst>
 </file>
@@ -407,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="52.77734375" customWidth="1"/>
@@ -470,6 +476,16 @@
         <v>12</v>
       </c>
     </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>